<commit_message>
feat(roster): add 5 permanent mock testing teams (155 total), admin credentials, and purge TECHTEAM10328
</commit_message>
<xml_diff>
--- a/data/participants_with_passwords.xlsx
+++ b/data/participants_with_passwords.xlsx
@@ -542,11 +542,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K223"/>
+  <dimension ref="A1:K233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="41" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -13269,6 +13269,576 @@
         </is>
       </c>
     </row>
+    <row r="224" ht="22" customHeight="1">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>TECHTEAM99001</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>Mock Team Alpha (Fresh)</t>
+        </is>
+      </c>
+      <c r="C224" s="4" t="inlineStr">
+        <is>
+          <t>99001</t>
+        </is>
+      </c>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>Mock Operator Alpha</t>
+        </is>
+      </c>
+      <c r="E224" s="5" t="inlineStr">
+        <is>
+          <t>Team Leader (PoC)</t>
+        </is>
+      </c>
+      <c r="F224" s="6" t="inlineStr">
+        <is>
+          <t>TLD-MOCK01</t>
+        </is>
+      </c>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>9999900001</t>
+        </is>
+      </c>
+      <c r="H224" s="3" t="inlineStr">
+        <is>
+          <t>mock.alpha1@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I224" s="3" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J224" s="7" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K224" s="3" t="inlineStr">
+        <is>
+          <t>TEST26001</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="22" customHeight="1">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>TECHTEAM99001</t>
+        </is>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>Mock Team Alpha (Fresh)</t>
+        </is>
+      </c>
+      <c r="C225" s="4" t="inlineStr">
+        <is>
+          <t>99002</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>Mock Partner Alpha</t>
+        </is>
+      </c>
+      <c r="E225" s="15" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F225" s="6" t="inlineStr">
+        <is>
+          <t>TLD-MOCK01</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>9999900002</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>mock.alpha2@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I225" s="3" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J225" s="7" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K225" s="3" t="inlineStr">
+        <is>
+          <t>TEST26002</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="22" customHeight="1">
+      <c r="A226" s="8" t="inlineStr">
+        <is>
+          <t>TECHTEAM99002</t>
+        </is>
+      </c>
+      <c r="B226" s="9" t="inlineStr">
+        <is>
+          <t>Mock Team Beta (Yellow Ready)</t>
+        </is>
+      </c>
+      <c r="C226" s="10" t="inlineStr">
+        <is>
+          <t>99003</t>
+        </is>
+      </c>
+      <c r="D226" s="9" t="inlineStr">
+        <is>
+          <t>Mock Operator Beta</t>
+        </is>
+      </c>
+      <c r="E226" s="14" t="inlineStr">
+        <is>
+          <t>Team Leader (PoC)</t>
+        </is>
+      </c>
+      <c r="F226" s="12" t="inlineStr">
+        <is>
+          <t>TLD-MOCK02</t>
+        </is>
+      </c>
+      <c r="G226" s="9" t="inlineStr">
+        <is>
+          <t>9999900003</t>
+        </is>
+      </c>
+      <c r="H226" s="9" t="inlineStr">
+        <is>
+          <t>mock.beta1@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I226" s="9" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J226" s="13" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K226" s="9" t="inlineStr">
+        <is>
+          <t>TEST26003</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="22" customHeight="1">
+      <c r="A227" s="8" t="inlineStr">
+        <is>
+          <t>TECHTEAM99002</t>
+        </is>
+      </c>
+      <c r="B227" s="9" t="inlineStr">
+        <is>
+          <t>Mock Team Beta (Yellow Ready)</t>
+        </is>
+      </c>
+      <c r="C227" s="10" t="inlineStr">
+        <is>
+          <t>99004</t>
+        </is>
+      </c>
+      <c r="D227" s="9" t="inlineStr">
+        <is>
+          <t>Mock Partner Beta</t>
+        </is>
+      </c>
+      <c r="E227" s="11" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F227" s="12" t="inlineStr">
+        <is>
+          <t>TLD-MOCK02</t>
+        </is>
+      </c>
+      <c r="G227" s="9" t="inlineStr">
+        <is>
+          <t>9999900004</t>
+        </is>
+      </c>
+      <c r="H227" s="9" t="inlineStr">
+        <is>
+          <t>mock.beta2@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I227" s="9" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J227" s="13" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K227" s="9" t="inlineStr">
+        <is>
+          <t>TEST26004</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="22" customHeight="1">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>TECHTEAM99003</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>Mock Team Gamma (Blue Ready)</t>
+        </is>
+      </c>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t>99005</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>Mock Operator Gamma</t>
+        </is>
+      </c>
+      <c r="E228" s="5" t="inlineStr">
+        <is>
+          <t>Team Leader (PoC)</t>
+        </is>
+      </c>
+      <c r="F228" s="6" t="inlineStr">
+        <is>
+          <t>TLD-MOCK03</t>
+        </is>
+      </c>
+      <c r="G228" s="3" t="inlineStr">
+        <is>
+          <t>9999900005</t>
+        </is>
+      </c>
+      <c r="H228" s="3" t="inlineStr">
+        <is>
+          <t>mock.gamma1@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I228" s="3" t="inlineStr">
+        <is>
+          <t>National Institute of Technology Karnataka</t>
+        </is>
+      </c>
+      <c r="J228" s="16" t="inlineStr">
+        <is>
+          <t>NONMAHE</t>
+        </is>
+      </c>
+      <c r="K228" s="3" t="inlineStr">
+        <is>
+          <t>TEST26005</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="22" customHeight="1">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>TECHTEAM99003</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>Mock Team Gamma (Blue Ready)</t>
+        </is>
+      </c>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t>99006</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>Mock Partner Gamma</t>
+        </is>
+      </c>
+      <c r="E229" s="15" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F229" s="6" t="inlineStr">
+        <is>
+          <t>TLD-MOCK03</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>9999900006</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>mock.gamma2@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I229" s="3" t="inlineStr">
+        <is>
+          <t>National Institute of Technology Karnataka</t>
+        </is>
+      </c>
+      <c r="J229" s="16" t="inlineStr">
+        <is>
+          <t>NONMAHE</t>
+        </is>
+      </c>
+      <c r="K229" s="3" t="inlineStr">
+        <is>
+          <t>TEST26006</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="22" customHeight="1">
+      <c r="A230" s="8" t="inlineStr">
+        <is>
+          <t>TECHTEAM99004</t>
+        </is>
+      </c>
+      <c r="B230" s="9" t="inlineStr">
+        <is>
+          <t>Mock Team Delta (Purple Ready)</t>
+        </is>
+      </c>
+      <c r="C230" s="10" t="inlineStr">
+        <is>
+          <t>99007</t>
+        </is>
+      </c>
+      <c r="D230" s="9" t="inlineStr">
+        <is>
+          <t>Mock Operator Delta</t>
+        </is>
+      </c>
+      <c r="E230" s="14" t="inlineStr">
+        <is>
+          <t>Team Leader (PoC)</t>
+        </is>
+      </c>
+      <c r="F230" s="12" t="inlineStr">
+        <is>
+          <t>TLD-MOCK04</t>
+        </is>
+      </c>
+      <c r="G230" s="9" t="inlineStr">
+        <is>
+          <t>9999900007</t>
+        </is>
+      </c>
+      <c r="H230" s="9" t="inlineStr">
+        <is>
+          <t>mock.delta1@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I230" s="9" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J230" s="13" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K230" s="9" t="inlineStr">
+        <is>
+          <t>TEST26007</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="22" customHeight="1">
+      <c r="A231" s="8" t="inlineStr">
+        <is>
+          <t>TECHTEAM99004</t>
+        </is>
+      </c>
+      <c r="B231" s="9" t="inlineStr">
+        <is>
+          <t>Mock Team Delta (Purple Ready)</t>
+        </is>
+      </c>
+      <c r="C231" s="10" t="inlineStr">
+        <is>
+          <t>99008</t>
+        </is>
+      </c>
+      <c r="D231" s="9" t="inlineStr">
+        <is>
+          <t>Mock Partner Delta</t>
+        </is>
+      </c>
+      <c r="E231" s="11" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F231" s="12" t="inlineStr">
+        <is>
+          <t>TLD-MOCK04</t>
+        </is>
+      </c>
+      <c r="G231" s="9" t="inlineStr">
+        <is>
+          <t>9999900008</t>
+        </is>
+      </c>
+      <c r="H231" s="9" t="inlineStr">
+        <is>
+          <t>mock.delta2@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I231" s="9" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J231" s="13" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K231" s="9" t="inlineStr">
+        <is>
+          <t>TEST26008</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="22" customHeight="1">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>TECHTEAM99005</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>Mock Team Omega (Survivor Cleared)</t>
+        </is>
+      </c>
+      <c r="C232" s="4" t="inlineStr">
+        <is>
+          <t>99009</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>Mock Operator Omega</t>
+        </is>
+      </c>
+      <c r="E232" s="5" t="inlineStr">
+        <is>
+          <t>Team Leader (PoC)</t>
+        </is>
+      </c>
+      <c r="F232" s="6" t="inlineStr">
+        <is>
+          <t>TLD-MOCK05</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>9999900009</t>
+        </is>
+      </c>
+      <c r="H232" s="3" t="inlineStr">
+        <is>
+          <t>mock.omega1@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I232" s="3" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J232" s="7" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K232" s="3" t="inlineStr">
+        <is>
+          <t>TEST26009</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="22" customHeight="1">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>TECHTEAM99005</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>Mock Team Omega (Survivor Cleared)</t>
+        </is>
+      </c>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>99010</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>Mock Partner Omega</t>
+        </is>
+      </c>
+      <c r="E233" s="15" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F233" s="6" t="inlineStr">
+        <is>
+          <t>TLD-MOCK05</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>9999900010</t>
+        </is>
+      </c>
+      <c r="H233" s="3" t="inlineStr">
+        <is>
+          <t>mock.omega2@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I233" s="3" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J233" s="7" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K233" s="3" t="inlineStr">
+        <is>
+          <t>TEST26010</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(mock): add 8 fresh mock test IDs at 0 points with admin visibility and self-healing
</commit_message>
<xml_diff>
--- a/data/participants_with_passwords.xlsx
+++ b/data/participants_with_passwords.xlsx
@@ -542,11 +542,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K233"/>
+  <dimension ref="A1:K239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="41" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -13287,7 +13287,7 @@
       </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
-          <t>Mock Operator Alpha</t>
+          <t>Mock Leader Alpha</t>
         </is>
       </c>
       <c r="E224" s="5" t="inlineStr">
@@ -13344,7 +13344,7 @@
       </c>
       <c r="D225" s="3" t="inlineStr">
         <is>
-          <t>Mock Partner Alpha</t>
+          <t>Mock Member Alpha</t>
         </is>
       </c>
       <c r="E225" s="15" t="inlineStr">
@@ -13391,7 +13391,7 @@
       </c>
       <c r="B226" s="9" t="inlineStr">
         <is>
-          <t>Mock Team Beta (Yellow Ready)</t>
+          <t>Mock Team Beta (Fresh)</t>
         </is>
       </c>
       <c r="C226" s="10" t="inlineStr">
@@ -13401,7 +13401,7 @@
       </c>
       <c r="D226" s="9" t="inlineStr">
         <is>
-          <t>Mock Operator Beta</t>
+          <t>Mock Leader Beta</t>
         </is>
       </c>
       <c r="E226" s="14" t="inlineStr">
@@ -13448,7 +13448,7 @@
       </c>
       <c r="B227" s="9" t="inlineStr">
         <is>
-          <t>Mock Team Beta (Yellow Ready)</t>
+          <t>Mock Team Beta (Fresh)</t>
         </is>
       </c>
       <c r="C227" s="10" t="inlineStr">
@@ -13458,7 +13458,7 @@
       </c>
       <c r="D227" s="9" t="inlineStr">
         <is>
-          <t>Mock Partner Beta</t>
+          <t>Mock Member Beta</t>
         </is>
       </c>
       <c r="E227" s="11" t="inlineStr">
@@ -13505,7 +13505,7 @@
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>Mock Team Gamma (Blue Ready)</t>
+          <t>Mock Team Gamma (Fresh)</t>
         </is>
       </c>
       <c r="C228" s="4" t="inlineStr">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
-          <t>Mock Operator Gamma</t>
+          <t>Mock Leader Gamma</t>
         </is>
       </c>
       <c r="E228" s="5" t="inlineStr">
@@ -13562,7 +13562,7 @@
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>Mock Team Gamma (Blue Ready)</t>
+          <t>Mock Team Gamma (Fresh)</t>
         </is>
       </c>
       <c r="C229" s="4" t="inlineStr">
@@ -13572,7 +13572,7 @@
       </c>
       <c r="D229" s="3" t="inlineStr">
         <is>
-          <t>Mock Partner Gamma</t>
+          <t>Mock Member Gamma</t>
         </is>
       </c>
       <c r="E229" s="15" t="inlineStr">
@@ -13619,7 +13619,7 @@
       </c>
       <c r="B230" s="9" t="inlineStr">
         <is>
-          <t>Mock Team Delta (Purple Ready)</t>
+          <t>Mock Team Delta (Fresh)</t>
         </is>
       </c>
       <c r="C230" s="10" t="inlineStr">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="D230" s="9" t="inlineStr">
         <is>
-          <t>Mock Operator Delta</t>
+          <t>Mock Leader Delta</t>
         </is>
       </c>
       <c r="E230" s="14" t="inlineStr">
@@ -13676,7 +13676,7 @@
       </c>
       <c r="B231" s="9" t="inlineStr">
         <is>
-          <t>Mock Team Delta (Purple Ready)</t>
+          <t>Mock Team Delta (Fresh)</t>
         </is>
       </c>
       <c r="C231" s="10" t="inlineStr">
@@ -13686,7 +13686,7 @@
       </c>
       <c r="D231" s="9" t="inlineStr">
         <is>
-          <t>Mock Partner Delta</t>
+          <t>Mock Member Delta</t>
         </is>
       </c>
       <c r="E231" s="11" t="inlineStr">
@@ -13733,7 +13733,7 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>Mock Team Omega (Survivor Cleared)</t>
+          <t>Mock Team Epsilon (Fresh)</t>
         </is>
       </c>
       <c r="C232" s="4" t="inlineStr">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
-          <t>Mock Operator Omega</t>
+          <t>Mock Leader Epsilon</t>
         </is>
       </c>
       <c r="E232" s="5" t="inlineStr">
@@ -13763,7 +13763,7 @@
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
-          <t>mock.omega1@techtatva.org</t>
+          <t>mock.epsilon1@techtatva.org</t>
         </is>
       </c>
       <c r="I232" s="3" t="inlineStr">
@@ -13790,7 +13790,7 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>Mock Team Omega (Survivor Cleared)</t>
+          <t>Mock Team Epsilon (Fresh)</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
@@ -13800,7 +13800,7 @@
       </c>
       <c r="D233" s="3" t="inlineStr">
         <is>
-          <t>Mock Partner Omega</t>
+          <t>Mock Member Epsilon</t>
         </is>
       </c>
       <c r="E233" s="15" t="inlineStr">
@@ -13820,7 +13820,7 @@
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>mock.omega2@techtatva.org</t>
+          <t>mock.epsilon2@techtatva.org</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
@@ -13836,6 +13836,348 @@
       <c r="K233" s="3" t="inlineStr">
         <is>
           <t>TEST26010</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="22" customHeight="1">
+      <c r="A234" s="8" t="inlineStr">
+        <is>
+          <t>TECHTEAM99006</t>
+        </is>
+      </c>
+      <c r="B234" s="9" t="inlineStr">
+        <is>
+          <t>Mock Team Zeta (Fresh)</t>
+        </is>
+      </c>
+      <c r="C234" s="10" t="inlineStr">
+        <is>
+          <t>99011</t>
+        </is>
+      </c>
+      <c r="D234" s="9" t="inlineStr">
+        <is>
+          <t>Mock Leader Zeta</t>
+        </is>
+      </c>
+      <c r="E234" s="14" t="inlineStr">
+        <is>
+          <t>Team Leader (PoC)</t>
+        </is>
+      </c>
+      <c r="F234" s="12" t="inlineStr">
+        <is>
+          <t>TLD-MOCK06</t>
+        </is>
+      </c>
+      <c r="G234" s="9" t="inlineStr">
+        <is>
+          <t>9999900011</t>
+        </is>
+      </c>
+      <c r="H234" s="9" t="inlineStr">
+        <is>
+          <t>mock.zeta1@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I234" s="9" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J234" s="13" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K234" s="9" t="inlineStr">
+        <is>
+          <t>TEST26011</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="22" customHeight="1">
+      <c r="A235" s="8" t="inlineStr">
+        <is>
+          <t>TECHTEAM99006</t>
+        </is>
+      </c>
+      <c r="B235" s="9" t="inlineStr">
+        <is>
+          <t>Mock Team Zeta (Fresh)</t>
+        </is>
+      </c>
+      <c r="C235" s="10" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="D235" s="9" t="inlineStr">
+        <is>
+          <t>Mock Member Zeta</t>
+        </is>
+      </c>
+      <c r="E235" s="11" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F235" s="12" t="inlineStr">
+        <is>
+          <t>TLD-MOCK06</t>
+        </is>
+      </c>
+      <c r="G235" s="9" t="inlineStr">
+        <is>
+          <t>9999900012</t>
+        </is>
+      </c>
+      <c r="H235" s="9" t="inlineStr">
+        <is>
+          <t>mock.zeta2@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I235" s="9" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J235" s="13" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K235" s="9" t="inlineStr">
+        <is>
+          <t>TEST26012</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="22" customHeight="1">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>TECHTEAM99007</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>Mock Team Eta (Fresh)</t>
+        </is>
+      </c>
+      <c r="C236" s="4" t="inlineStr">
+        <is>
+          <t>99013</t>
+        </is>
+      </c>
+      <c r="D236" s="3" t="inlineStr">
+        <is>
+          <t>Mock Leader Eta</t>
+        </is>
+      </c>
+      <c r="E236" s="5" t="inlineStr">
+        <is>
+          <t>Team Leader (PoC)</t>
+        </is>
+      </c>
+      <c r="F236" s="6" t="inlineStr">
+        <is>
+          <t>TLD-MOCK07</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="inlineStr">
+        <is>
+          <t>9999900013</t>
+        </is>
+      </c>
+      <c r="H236" s="3" t="inlineStr">
+        <is>
+          <t>mock.eta1@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I236" s="3" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J236" s="7" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K236" s="3" t="inlineStr">
+        <is>
+          <t>TEST26013</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="22" customHeight="1">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>TECHTEAM99007</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>Mock Team Eta (Fresh)</t>
+        </is>
+      </c>
+      <c r="C237" s="4" t="inlineStr">
+        <is>
+          <t>99014</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="inlineStr">
+        <is>
+          <t>Mock Member Eta</t>
+        </is>
+      </c>
+      <c r="E237" s="15" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F237" s="6" t="inlineStr">
+        <is>
+          <t>TLD-MOCK07</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="inlineStr">
+        <is>
+          <t>9999900014</t>
+        </is>
+      </c>
+      <c r="H237" s="3" t="inlineStr">
+        <is>
+          <t>mock.eta2@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I237" s="3" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J237" s="7" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K237" s="3" t="inlineStr">
+        <is>
+          <t>TEST26014</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="22" customHeight="1">
+      <c r="A238" s="8" t="inlineStr">
+        <is>
+          <t>TECHTEAM99008</t>
+        </is>
+      </c>
+      <c r="B238" s="9" t="inlineStr">
+        <is>
+          <t>Mock Team Theta (Fresh)</t>
+        </is>
+      </c>
+      <c r="C238" s="10" t="inlineStr">
+        <is>
+          <t>99015</t>
+        </is>
+      </c>
+      <c r="D238" s="9" t="inlineStr">
+        <is>
+          <t>Mock Leader Theta</t>
+        </is>
+      </c>
+      <c r="E238" s="14" t="inlineStr">
+        <is>
+          <t>Team Leader (PoC)</t>
+        </is>
+      </c>
+      <c r="F238" s="12" t="inlineStr">
+        <is>
+          <t>TLD-MOCK08</t>
+        </is>
+      </c>
+      <c r="G238" s="9" t="inlineStr">
+        <is>
+          <t>9999900015</t>
+        </is>
+      </c>
+      <c r="H238" s="9" t="inlineStr">
+        <is>
+          <t>mock.theta1@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I238" s="9" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J238" s="13" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K238" s="9" t="inlineStr">
+        <is>
+          <t>TEST26015</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="22" customHeight="1">
+      <c r="A239" s="8" t="inlineStr">
+        <is>
+          <t>TECHTEAM99008</t>
+        </is>
+      </c>
+      <c r="B239" s="9" t="inlineStr">
+        <is>
+          <t>Mock Team Theta (Fresh)</t>
+        </is>
+      </c>
+      <c r="C239" s="10" t="inlineStr">
+        <is>
+          <t>99016</t>
+        </is>
+      </c>
+      <c r="D239" s="9" t="inlineStr">
+        <is>
+          <t>Mock Member Theta</t>
+        </is>
+      </c>
+      <c r="E239" s="11" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F239" s="12" t="inlineStr">
+        <is>
+          <t>TLD-MOCK08</t>
+        </is>
+      </c>
+      <c r="G239" s="9" t="inlineStr">
+        <is>
+          <t>9999900016</t>
+        </is>
+      </c>
+      <c r="H239" s="9" t="inlineStr">
+        <is>
+          <t>mock.theta2@techtatva.org</t>
+        </is>
+      </c>
+      <c r="I239" s="9" t="inlineStr">
+        <is>
+          <t>Manipal Institute of Technology</t>
+        </is>
+      </c>
+      <c r="J239" s="13" t="inlineStr">
+        <is>
+          <t>MAHE</t>
+        </is>
+      </c>
+      <c r="K239" s="9" t="inlineStr">
+        <is>
+          <t>TEST26016</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
security: remove all mock test IDs and delete master answer key before live event
</commit_message>
<xml_diff>
--- a/data/participants_with_passwords.xlsx
+++ b/data/participants_with_passwords.xlsx
@@ -542,11 +542,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K239"/>
+  <dimension ref="A1:K223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="41" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -13269,918 +13269,6 @@
         </is>
       </c>
     </row>
-    <row r="224" ht="22" customHeight="1">
-      <c r="A224" s="2" t="inlineStr">
-        <is>
-          <t>TECHTEAM99001</t>
-        </is>
-      </c>
-      <c r="B224" s="3" t="inlineStr">
-        <is>
-          <t>Mock Team Alpha (Fresh)</t>
-        </is>
-      </c>
-      <c r="C224" s="4" t="inlineStr">
-        <is>
-          <t>99001</t>
-        </is>
-      </c>
-      <c r="D224" s="3" t="inlineStr">
-        <is>
-          <t>Mock Leader Alpha</t>
-        </is>
-      </c>
-      <c r="E224" s="5" t="inlineStr">
-        <is>
-          <t>Team Leader (PoC)</t>
-        </is>
-      </c>
-      <c r="F224" s="6" t="inlineStr">
-        <is>
-          <t>TLD-MOCK01</t>
-        </is>
-      </c>
-      <c r="G224" s="3" t="inlineStr">
-        <is>
-          <t>9999900001</t>
-        </is>
-      </c>
-      <c r="H224" s="3" t="inlineStr">
-        <is>
-          <t>mock.alpha1@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I224" s="3" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J224" s="7" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K224" s="3" t="inlineStr">
-        <is>
-          <t>TEST26001</t>
-        </is>
-      </c>
-    </row>
-    <row r="225" ht="22" customHeight="1">
-      <c r="A225" s="2" t="inlineStr">
-        <is>
-          <t>TECHTEAM99001</t>
-        </is>
-      </c>
-      <c r="B225" s="3" t="inlineStr">
-        <is>
-          <t>Mock Team Alpha (Fresh)</t>
-        </is>
-      </c>
-      <c r="C225" s="4" t="inlineStr">
-        <is>
-          <t>99002</t>
-        </is>
-      </c>
-      <c r="D225" s="3" t="inlineStr">
-        <is>
-          <t>Mock Member Alpha</t>
-        </is>
-      </c>
-      <c r="E225" s="15" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="F225" s="6" t="inlineStr">
-        <is>
-          <t>TLD-MOCK01</t>
-        </is>
-      </c>
-      <c r="G225" s="3" t="inlineStr">
-        <is>
-          <t>9999900002</t>
-        </is>
-      </c>
-      <c r="H225" s="3" t="inlineStr">
-        <is>
-          <t>mock.alpha2@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I225" s="3" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J225" s="7" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K225" s="3" t="inlineStr">
-        <is>
-          <t>TEST26002</t>
-        </is>
-      </c>
-    </row>
-    <row r="226" ht="22" customHeight="1">
-      <c r="A226" s="8" t="inlineStr">
-        <is>
-          <t>TECHTEAM99002</t>
-        </is>
-      </c>
-      <c r="B226" s="9" t="inlineStr">
-        <is>
-          <t>Mock Team Beta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C226" s="10" t="inlineStr">
-        <is>
-          <t>99003</t>
-        </is>
-      </c>
-      <c r="D226" s="9" t="inlineStr">
-        <is>
-          <t>Mock Leader Beta</t>
-        </is>
-      </c>
-      <c r="E226" s="14" t="inlineStr">
-        <is>
-          <t>Team Leader (PoC)</t>
-        </is>
-      </c>
-      <c r="F226" s="12" t="inlineStr">
-        <is>
-          <t>TLD-MOCK02</t>
-        </is>
-      </c>
-      <c r="G226" s="9" t="inlineStr">
-        <is>
-          <t>9999900003</t>
-        </is>
-      </c>
-      <c r="H226" s="9" t="inlineStr">
-        <is>
-          <t>mock.beta1@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I226" s="9" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J226" s="13" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K226" s="9" t="inlineStr">
-        <is>
-          <t>TEST26003</t>
-        </is>
-      </c>
-    </row>
-    <row r="227" ht="22" customHeight="1">
-      <c r="A227" s="8" t="inlineStr">
-        <is>
-          <t>TECHTEAM99002</t>
-        </is>
-      </c>
-      <c r="B227" s="9" t="inlineStr">
-        <is>
-          <t>Mock Team Beta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C227" s="10" t="inlineStr">
-        <is>
-          <t>99004</t>
-        </is>
-      </c>
-      <c r="D227" s="9" t="inlineStr">
-        <is>
-          <t>Mock Member Beta</t>
-        </is>
-      </c>
-      <c r="E227" s="11" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="F227" s="12" t="inlineStr">
-        <is>
-          <t>TLD-MOCK02</t>
-        </is>
-      </c>
-      <c r="G227" s="9" t="inlineStr">
-        <is>
-          <t>9999900004</t>
-        </is>
-      </c>
-      <c r="H227" s="9" t="inlineStr">
-        <is>
-          <t>mock.beta2@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I227" s="9" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J227" s="13" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K227" s="9" t="inlineStr">
-        <is>
-          <t>TEST26004</t>
-        </is>
-      </c>
-    </row>
-    <row r="228" ht="22" customHeight="1">
-      <c r="A228" s="2" t="inlineStr">
-        <is>
-          <t>TECHTEAM99003</t>
-        </is>
-      </c>
-      <c r="B228" s="3" t="inlineStr">
-        <is>
-          <t>Mock Team Gamma (Fresh)</t>
-        </is>
-      </c>
-      <c r="C228" s="4" t="inlineStr">
-        <is>
-          <t>99005</t>
-        </is>
-      </c>
-      <c r="D228" s="3" t="inlineStr">
-        <is>
-          <t>Mock Leader Gamma</t>
-        </is>
-      </c>
-      <c r="E228" s="5" t="inlineStr">
-        <is>
-          <t>Team Leader (PoC)</t>
-        </is>
-      </c>
-      <c r="F228" s="6" t="inlineStr">
-        <is>
-          <t>TLD-MOCK03</t>
-        </is>
-      </c>
-      <c r="G228" s="3" t="inlineStr">
-        <is>
-          <t>9999900005</t>
-        </is>
-      </c>
-      <c r="H228" s="3" t="inlineStr">
-        <is>
-          <t>mock.gamma1@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I228" s="3" t="inlineStr">
-        <is>
-          <t>National Institute of Technology Karnataka</t>
-        </is>
-      </c>
-      <c r="J228" s="16" t="inlineStr">
-        <is>
-          <t>NONMAHE</t>
-        </is>
-      </c>
-      <c r="K228" s="3" t="inlineStr">
-        <is>
-          <t>TEST26005</t>
-        </is>
-      </c>
-    </row>
-    <row r="229" ht="22" customHeight="1">
-      <c r="A229" s="2" t="inlineStr">
-        <is>
-          <t>TECHTEAM99003</t>
-        </is>
-      </c>
-      <c r="B229" s="3" t="inlineStr">
-        <is>
-          <t>Mock Team Gamma (Fresh)</t>
-        </is>
-      </c>
-      <c r="C229" s="4" t="inlineStr">
-        <is>
-          <t>99006</t>
-        </is>
-      </c>
-      <c r="D229" s="3" t="inlineStr">
-        <is>
-          <t>Mock Member Gamma</t>
-        </is>
-      </c>
-      <c r="E229" s="15" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="F229" s="6" t="inlineStr">
-        <is>
-          <t>TLD-MOCK03</t>
-        </is>
-      </c>
-      <c r="G229" s="3" t="inlineStr">
-        <is>
-          <t>9999900006</t>
-        </is>
-      </c>
-      <c r="H229" s="3" t="inlineStr">
-        <is>
-          <t>mock.gamma2@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I229" s="3" t="inlineStr">
-        <is>
-          <t>National Institute of Technology Karnataka</t>
-        </is>
-      </c>
-      <c r="J229" s="16" t="inlineStr">
-        <is>
-          <t>NONMAHE</t>
-        </is>
-      </c>
-      <c r="K229" s="3" t="inlineStr">
-        <is>
-          <t>TEST26006</t>
-        </is>
-      </c>
-    </row>
-    <row r="230" ht="22" customHeight="1">
-      <c r="A230" s="8" t="inlineStr">
-        <is>
-          <t>TECHTEAM99004</t>
-        </is>
-      </c>
-      <c r="B230" s="9" t="inlineStr">
-        <is>
-          <t>Mock Team Delta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C230" s="10" t="inlineStr">
-        <is>
-          <t>99007</t>
-        </is>
-      </c>
-      <c r="D230" s="9" t="inlineStr">
-        <is>
-          <t>Mock Leader Delta</t>
-        </is>
-      </c>
-      <c r="E230" s="14" t="inlineStr">
-        <is>
-          <t>Team Leader (PoC)</t>
-        </is>
-      </c>
-      <c r="F230" s="12" t="inlineStr">
-        <is>
-          <t>TLD-MOCK04</t>
-        </is>
-      </c>
-      <c r="G230" s="9" t="inlineStr">
-        <is>
-          <t>9999900007</t>
-        </is>
-      </c>
-      <c r="H230" s="9" t="inlineStr">
-        <is>
-          <t>mock.delta1@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I230" s="9" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J230" s="13" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K230" s="9" t="inlineStr">
-        <is>
-          <t>TEST26007</t>
-        </is>
-      </c>
-    </row>
-    <row r="231" ht="22" customHeight="1">
-      <c r="A231" s="8" t="inlineStr">
-        <is>
-          <t>TECHTEAM99004</t>
-        </is>
-      </c>
-      <c r="B231" s="9" t="inlineStr">
-        <is>
-          <t>Mock Team Delta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C231" s="10" t="inlineStr">
-        <is>
-          <t>99008</t>
-        </is>
-      </c>
-      <c r="D231" s="9" t="inlineStr">
-        <is>
-          <t>Mock Member Delta</t>
-        </is>
-      </c>
-      <c r="E231" s="11" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="F231" s="12" t="inlineStr">
-        <is>
-          <t>TLD-MOCK04</t>
-        </is>
-      </c>
-      <c r="G231" s="9" t="inlineStr">
-        <is>
-          <t>9999900008</t>
-        </is>
-      </c>
-      <c r="H231" s="9" t="inlineStr">
-        <is>
-          <t>mock.delta2@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I231" s="9" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J231" s="13" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K231" s="9" t="inlineStr">
-        <is>
-          <t>TEST26008</t>
-        </is>
-      </c>
-    </row>
-    <row r="232" ht="22" customHeight="1">
-      <c r="A232" s="2" t="inlineStr">
-        <is>
-          <t>TECHTEAM99005</t>
-        </is>
-      </c>
-      <c r="B232" s="3" t="inlineStr">
-        <is>
-          <t>Mock Team Epsilon (Fresh)</t>
-        </is>
-      </c>
-      <c r="C232" s="4" t="inlineStr">
-        <is>
-          <t>99009</t>
-        </is>
-      </c>
-      <c r="D232" s="3" t="inlineStr">
-        <is>
-          <t>Mock Leader Epsilon</t>
-        </is>
-      </c>
-      <c r="E232" s="5" t="inlineStr">
-        <is>
-          <t>Team Leader (PoC)</t>
-        </is>
-      </c>
-      <c r="F232" s="6" t="inlineStr">
-        <is>
-          <t>TLD-MOCK05</t>
-        </is>
-      </c>
-      <c r="G232" s="3" t="inlineStr">
-        <is>
-          <t>9999900009</t>
-        </is>
-      </c>
-      <c r="H232" s="3" t="inlineStr">
-        <is>
-          <t>mock.epsilon1@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I232" s="3" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J232" s="7" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K232" s="3" t="inlineStr">
-        <is>
-          <t>TEST26009</t>
-        </is>
-      </c>
-    </row>
-    <row r="233" ht="22" customHeight="1">
-      <c r="A233" s="2" t="inlineStr">
-        <is>
-          <t>TECHTEAM99005</t>
-        </is>
-      </c>
-      <c r="B233" s="3" t="inlineStr">
-        <is>
-          <t>Mock Team Epsilon (Fresh)</t>
-        </is>
-      </c>
-      <c r="C233" s="4" t="inlineStr">
-        <is>
-          <t>99010</t>
-        </is>
-      </c>
-      <c r="D233" s="3" t="inlineStr">
-        <is>
-          <t>Mock Member Epsilon</t>
-        </is>
-      </c>
-      <c r="E233" s="15" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="F233" s="6" t="inlineStr">
-        <is>
-          <t>TLD-MOCK05</t>
-        </is>
-      </c>
-      <c r="G233" s="3" t="inlineStr">
-        <is>
-          <t>9999900010</t>
-        </is>
-      </c>
-      <c r="H233" s="3" t="inlineStr">
-        <is>
-          <t>mock.epsilon2@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I233" s="3" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J233" s="7" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K233" s="3" t="inlineStr">
-        <is>
-          <t>TEST26010</t>
-        </is>
-      </c>
-    </row>
-    <row r="234" ht="22" customHeight="1">
-      <c r="A234" s="8" t="inlineStr">
-        <is>
-          <t>TECHTEAM99006</t>
-        </is>
-      </c>
-      <c r="B234" s="9" t="inlineStr">
-        <is>
-          <t>Mock Team Zeta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C234" s="10" t="inlineStr">
-        <is>
-          <t>99011</t>
-        </is>
-      </c>
-      <c r="D234" s="9" t="inlineStr">
-        <is>
-          <t>Mock Leader Zeta</t>
-        </is>
-      </c>
-      <c r="E234" s="14" t="inlineStr">
-        <is>
-          <t>Team Leader (PoC)</t>
-        </is>
-      </c>
-      <c r="F234" s="12" t="inlineStr">
-        <is>
-          <t>TLD-MOCK06</t>
-        </is>
-      </c>
-      <c r="G234" s="9" t="inlineStr">
-        <is>
-          <t>9999900011</t>
-        </is>
-      </c>
-      <c r="H234" s="9" t="inlineStr">
-        <is>
-          <t>mock.zeta1@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I234" s="9" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J234" s="13" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K234" s="9" t="inlineStr">
-        <is>
-          <t>TEST26011</t>
-        </is>
-      </c>
-    </row>
-    <row r="235" ht="22" customHeight="1">
-      <c r="A235" s="8" t="inlineStr">
-        <is>
-          <t>TECHTEAM99006</t>
-        </is>
-      </c>
-      <c r="B235" s="9" t="inlineStr">
-        <is>
-          <t>Mock Team Zeta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C235" s="10" t="inlineStr">
-        <is>
-          <t>99012</t>
-        </is>
-      </c>
-      <c r="D235" s="9" t="inlineStr">
-        <is>
-          <t>Mock Member Zeta</t>
-        </is>
-      </c>
-      <c r="E235" s="11" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="F235" s="12" t="inlineStr">
-        <is>
-          <t>TLD-MOCK06</t>
-        </is>
-      </c>
-      <c r="G235" s="9" t="inlineStr">
-        <is>
-          <t>9999900012</t>
-        </is>
-      </c>
-      <c r="H235" s="9" t="inlineStr">
-        <is>
-          <t>mock.zeta2@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I235" s="9" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J235" s="13" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K235" s="9" t="inlineStr">
-        <is>
-          <t>TEST26012</t>
-        </is>
-      </c>
-    </row>
-    <row r="236" ht="22" customHeight="1">
-      <c r="A236" s="2" t="inlineStr">
-        <is>
-          <t>TECHTEAM99007</t>
-        </is>
-      </c>
-      <c r="B236" s="3" t="inlineStr">
-        <is>
-          <t>Mock Team Eta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C236" s="4" t="inlineStr">
-        <is>
-          <t>99013</t>
-        </is>
-      </c>
-      <c r="D236" s="3" t="inlineStr">
-        <is>
-          <t>Mock Leader Eta</t>
-        </is>
-      </c>
-      <c r="E236" s="5" t="inlineStr">
-        <is>
-          <t>Team Leader (PoC)</t>
-        </is>
-      </c>
-      <c r="F236" s="6" t="inlineStr">
-        <is>
-          <t>TLD-MOCK07</t>
-        </is>
-      </c>
-      <c r="G236" s="3" t="inlineStr">
-        <is>
-          <t>9999900013</t>
-        </is>
-      </c>
-      <c r="H236" s="3" t="inlineStr">
-        <is>
-          <t>mock.eta1@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I236" s="3" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J236" s="7" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K236" s="3" t="inlineStr">
-        <is>
-          <t>TEST26013</t>
-        </is>
-      </c>
-    </row>
-    <row r="237" ht="22" customHeight="1">
-      <c r="A237" s="2" t="inlineStr">
-        <is>
-          <t>TECHTEAM99007</t>
-        </is>
-      </c>
-      <c r="B237" s="3" t="inlineStr">
-        <is>
-          <t>Mock Team Eta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C237" s="4" t="inlineStr">
-        <is>
-          <t>99014</t>
-        </is>
-      </c>
-      <c r="D237" s="3" t="inlineStr">
-        <is>
-          <t>Mock Member Eta</t>
-        </is>
-      </c>
-      <c r="E237" s="15" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="F237" s="6" t="inlineStr">
-        <is>
-          <t>TLD-MOCK07</t>
-        </is>
-      </c>
-      <c r="G237" s="3" t="inlineStr">
-        <is>
-          <t>9999900014</t>
-        </is>
-      </c>
-      <c r="H237" s="3" t="inlineStr">
-        <is>
-          <t>mock.eta2@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I237" s="3" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J237" s="7" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K237" s="3" t="inlineStr">
-        <is>
-          <t>TEST26014</t>
-        </is>
-      </c>
-    </row>
-    <row r="238" ht="22" customHeight="1">
-      <c r="A238" s="8" t="inlineStr">
-        <is>
-          <t>TECHTEAM99008</t>
-        </is>
-      </c>
-      <c r="B238" s="9" t="inlineStr">
-        <is>
-          <t>Mock Team Theta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C238" s="10" t="inlineStr">
-        <is>
-          <t>99015</t>
-        </is>
-      </c>
-      <c r="D238" s="9" t="inlineStr">
-        <is>
-          <t>Mock Leader Theta</t>
-        </is>
-      </c>
-      <c r="E238" s="14" t="inlineStr">
-        <is>
-          <t>Team Leader (PoC)</t>
-        </is>
-      </c>
-      <c r="F238" s="12" t="inlineStr">
-        <is>
-          <t>TLD-MOCK08</t>
-        </is>
-      </c>
-      <c r="G238" s="9" t="inlineStr">
-        <is>
-          <t>9999900015</t>
-        </is>
-      </c>
-      <c r="H238" s="9" t="inlineStr">
-        <is>
-          <t>mock.theta1@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I238" s="9" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J238" s="13" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K238" s="9" t="inlineStr">
-        <is>
-          <t>TEST26015</t>
-        </is>
-      </c>
-    </row>
-    <row r="239" ht="22" customHeight="1">
-      <c r="A239" s="8" t="inlineStr">
-        <is>
-          <t>TECHTEAM99008</t>
-        </is>
-      </c>
-      <c r="B239" s="9" t="inlineStr">
-        <is>
-          <t>Mock Team Theta (Fresh)</t>
-        </is>
-      </c>
-      <c r="C239" s="10" t="inlineStr">
-        <is>
-          <t>99016</t>
-        </is>
-      </c>
-      <c r="D239" s="9" t="inlineStr">
-        <is>
-          <t>Mock Member Theta</t>
-        </is>
-      </c>
-      <c r="E239" s="11" t="inlineStr">
-        <is>
-          <t>Member</t>
-        </is>
-      </c>
-      <c r="F239" s="12" t="inlineStr">
-        <is>
-          <t>TLD-MOCK08</t>
-        </is>
-      </c>
-      <c r="G239" s="9" t="inlineStr">
-        <is>
-          <t>9999900016</t>
-        </is>
-      </c>
-      <c r="H239" s="9" t="inlineStr">
-        <is>
-          <t>mock.theta2@techtatva.org</t>
-        </is>
-      </c>
-      <c r="I239" s="9" t="inlineStr">
-        <is>
-          <t>Manipal Institute of Technology</t>
-        </is>
-      </c>
-      <c r="J239" s="13" t="inlineStr">
-        <is>
-          <t>MAHE</t>
-        </is>
-      </c>
-      <c r="K239" s="9" t="inlineStr">
-        <is>
-          <t>TEST26016</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>